<commit_message>
chore: sync automatico fim de sessao 2026-09-10
</commit_message>
<xml_diff>
--- a/docs/fluxo-victoria-2026-09-10.xlsx
+++ b/docs/fluxo-victoria-2026-09-10.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etapas Evo" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Itens'!$A$1:$I$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Itens'!$A$1:$I$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Etapas Evo'!$A$1:$G$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -773,7 +773,7 @@
         <v>2</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>3</v>
@@ -1326,7 +1326,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="327" customHeight="1">
+    <row r="3" ht="336" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>VictorIA</t>
@@ -1348,7 +1348,7 @@
 • CNPJ chega → checagens automáticas (ver Sistemas): DV inválido / não consta na Receita → NÃO pré-aprova
 • CNPJ já na base AIVA/Odres → mensagem oficial + transfere pro funil 19 (tag ODRES/UME)
 • CNPJ &lt; 1 ano → NAO_QUALIFICADO + card vai pra 93
-• Sem sócio na Receita (QSA vazio) → tag SEM_SOCIO → fluxo dos 5 documentos (Drive)
+• Sem sócio na Receita (QSA vazio) → segue igual a qualquer lead (regra 10/09: sem documentos, sem tag)
 • Objeções, taxa 12% × juros do cliente, nunca simula parcelas, nunca acusa golpe
 • 7 dados completos → PRE_APROVACAO + aciona humano (qualificacao_inicial_completa)</t>
         </is>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="J4" s="13" t="inlineStr"/>
     </row>
-    <row r="5" ht="227" customHeight="1">
+    <row r="5" ht="196" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Rotinas automáticas</t>
@@ -1488,8 +1488,7 @@
 • reativação 10h: parado 48h–14d → HSM 48 (20/execução)
 • reengajamento 16h seg–sex: follow-up personalizado via HSM 48, até 3× a cada 15d
 • régua-saída 10h30: 3 reengajamentos + 15d mudo + bola com o lead → card 53 + SEM_RESPOSTA
-• auto-descarte: INTERESSADO +21d sem msg do lead → AGUARDANDO
-• cobrança-docs 10h: sem sócio parado 2d+ → lembrete HSM 48 (máx 3)</t>
+• auto-descarte: INTERESSADO +21d sem msg do lead → AGUARDANDO</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -1621,7 +1620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I116"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2226,7 +2225,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Sem sócio na Receita (QSA vazio) → tag SEM_SOCIO → fluxo dos 5 documentos (Drive)</t>
+          <t>Sem sócio na Receita (QSA vazio) → segue igual a qualquer lead (regra 10/09: sem documentos, sem tag)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
@@ -2506,17 +2505,17 @@
       <c r="C30" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="D30" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>cobrança-docs 10h: sem sócio parado 2d+ → lembrete HSM 48 (máx 3)</t>
+          <t>BrasilAPI (Receita): idade, situação, QSA — marcador [CNPJ_RECEITA] impede revalidar</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr"/>
@@ -2541,11 +2540,11 @@
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>BrasilAPI (Receita): idade, situação, QSA — marcador [CNPJ_RECEITA] impede revalidar</t>
+          <t>aiva_base_cnpjs (6.323 CNPJs, importada 11h todo dia via Data Studio)</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr"/>
@@ -2570,11 +2569,11 @@
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>aiva_base_cnpjs (6.323 CNPJs, importada 11h todo dia via Data Studio)</t>
+          <t>sdr_registros_cnpj (status informada) · formsdata da opp no Evo</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
@@ -2583,27 +2582,27 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Interessado</t>
+          <t>Pré Aprovação</t>
         </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="D33" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>54</v>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>sdr_registros_cnpj (status informada) · formsdata da opp no Evo</t>
+          <t>FASE 2 — só tranquiliza: "estamos analisando, em breve retorno". Não pede dado, não promete prazo</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
@@ -2628,11 +2627,11 @@
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>FASE 2 — só tranquiliza: "estamos analisando, em breve retorno". Não pede dado, não promete prazo</t>
+          <t>Se o CNPJ tiver ≥ 3 lojas → tag IMPORTANTE (74) na opp</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr"/>
@@ -2657,11 +2656,11 @@
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Se o CNPJ tiver ≥ 3 lojas → tag IMPORTANTE (74) na opp</t>
+          <t>Alerta Nei + Aldo: pré-aprovação enviada</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr"/>
@@ -2680,17 +2679,17 @@
       <c r="C36" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D36" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Alerta Nei + Aldo: pré-aprovação enviada</t>
+          <t>Edu (AIVA) analisa a pré-aprovação pela planilha, em até 24h</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr"/>
@@ -2715,11 +2714,11 @@
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Edu (AIVA) analisa a pré-aprovação pela planilha, em até 24h</t>
+          <t>Aprovou → Nei move o card 54 → 49 (Cadastro Recebido)</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr"/>
@@ -2744,11 +2743,11 @@
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Aprovou → Nei move o card 54 → 49 (Cadastro Recebido)</t>
+          <t>Reprovou → descarte (Nei marca no Evo)</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr"/>
@@ -2767,17 +2766,17 @@
       <c r="C39" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D39" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Reprovou → descarte (Nei marca no Evo)</t>
+          <t>Nenhuma cobrança automática nessa etapa (espera humana)</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr"/>
@@ -2796,9 +2795,9 @@
       <c r="C40" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D40" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
@@ -2806,7 +2805,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Nenhuma cobrança automática nessa etapa (espera humana)</t>
+          <t>Planilha AIVA APROVAÇÃO (Google Sheets) — linha por lead pré-aprovado</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr"/>
@@ -2831,11 +2830,11 @@
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Planilha AIVA APROVAÇÃO (Google Sheets) — linha por lead pré-aprovado</t>
+          <t>Tags Evo: AIVA (69) sempre · IMPORTANTE (74) se ≥ 3 lojas</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr"/>
@@ -2844,27 +2843,27 @@
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Pré Aprovação</t>
+          <t>Cadastro Recebido</t>
         </is>
       </c>
       <c r="C42" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="D42" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>49</v>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Tags Evo: AIVA (69) sempre · IMPORTANTE (74) se ≥ 3 lojas</t>
+          <t>Entrada na etapa → HSM 29 "Complete o cadastro" reabre a janela; status volta a INTERESSADO com marcador de Fase 3</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr"/>
@@ -2889,11 +2888,11 @@
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → HSM 29 "Complete o cadastro" reabre a janela; status volta a INTERESSADO com marcador de Fase 3</t>
+          <t>FASE 3 — coleta 5 dados: e-mail do sócio · faturamento anual · boleto mensal · localização das lojas · CNPJs adicionais (só se ≥ 2 lojas)</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr"/>
@@ -2918,11 +2917,11 @@
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>FASE 3 — coleta 5 dados: e-mail do sócio · faturamento anual · boleto mensal · localização das lojas · CNPJs adicionais (só se ≥ 2 lojas)</t>
+          <t>Dados sensíveis: explica o porquê, aceita "por alto"; recusa → aciona humano (receio_dados_sensiveis)</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr"/>
@@ -2947,11 +2946,11 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Dados sensíveis: explica o porquê, aceita "por alto"; recusa → aciona humano (receio_dados_sensiveis)</t>
+          <t>Trava anti-conclusão: sem os 5, nunca diz "cadastro completo"</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr"/>
@@ -2976,11 +2975,11 @@
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Trava anti-conclusão: sem os 5, nunca diz "cadastro completo"</t>
+          <t>12 dados completos → CADASTRO_RECEBIDO + HubSpot + registro do CNPJ + alerta ✅ (cadastro_completo)</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr"/>
@@ -2999,17 +2998,17 @@
       <c r="C47" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D47" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>12 dados completos → CADASTRO_RECEBIDO + HubSpot + registro do CNPJ + alerta ✅ (cadastro_completo)</t>
+          <t>Nei confere no /registros e move o card 49 → 50 (Em Análise)</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr"/>
@@ -3034,11 +3033,11 @@
         </is>
       </c>
       <c r="E48" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Nei confere no /registros e move o card 49 → 50 (Em Análise)</t>
+          <t>Cobrança esgotada (3 toques) → escala pro Nei uma vez</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr"/>
@@ -3057,17 +3056,17 @@
       <c r="C49" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D49" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Cobrança esgotada (3 toques) → escala pro Nei uma vez</t>
+          <t>cadastro-recebido-cobranca 15h seg–sex: D+1 · D+3 · D+7 na etapa → HSM 48 + pede o dado que falta (um por vez)</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr"/>
@@ -3092,11 +3091,11 @@
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>cadastro-recebido-cobranca 15h seg–sex: D+1 · D+3 · D+7 na etapa → HSM 48 + pede o dado que falta (um por vez)</t>
+          <t>Fonte da verdade = etapa do Evo (stagebegintime)</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr"/>
@@ -3115,17 +3114,17 @@
       <c r="C51" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D51" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Fonte da verdade = etapa do Evo (stagebegintime)</t>
+          <t>HubSpot (contato/empresa) — só quando os 12 dados fecham</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr"/>
@@ -3150,11 +3149,11 @@
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>HubSpot (contato/empresa) — só quando os 12 dados fecham</t>
+          <t>sdr_registros_cnpj (matriz + adicionais) · formsdata da opp</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr"/>
@@ -3179,11 +3178,11 @@
         </is>
       </c>
       <c r="E53" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>sdr_registros_cnpj (matriz + adicionais) · formsdata da opp</t>
+          <t>Painel /registros</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr"/>
@@ -3192,27 +3191,27 @@
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Cadastro Recebido</t>
+          <t>Em Análise AIVA</t>
         </is>
       </c>
       <c r="C54" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="D54" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>50</v>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Painel /registros</t>
+          <t>Entrada na etapa → HSM 34 (aprovação) com o link do onboarding retail-onboarding-hub + biometria (CAF)</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr"/>
@@ -3237,11 +3236,11 @@
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → HSM 34 (aprovação) com o link do onboarding retail-onboarding-hub + biometria (CAF)</t>
+          <t>FASE 4 — acompanha: "conseguiu acessar? concluiu a biometria?"</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr"/>
@@ -3266,11 +3265,11 @@
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>FASE 4 — acompanha: "conseguiu acessar? concluiu a biometria?"</t>
+          <t>Qualquer erro → PEDE O PRINT primeiro (regra 08/09) · dificuldade → aciona humano (dificuldade_onboarding_caf)</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr"/>
@@ -3295,11 +3294,11 @@
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Qualquer erro → PEDE O PRINT primeiro (regra 08/09) · dificuldade → aciona humano (dificuldade_onboarding_caf)</t>
+          <t>Lead diz que concluiu → aciona humano (cadastro_caf_confirmado)</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr"/>
@@ -3324,11 +3323,11 @@
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Lead diz que concluiu → aciona humano (cadastro_caf_confirmado)</t>
+          <t>Nunca reenvia o link sozinha; status fica EM_ANALISE_AIVA (só o time muda)</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr"/>
@@ -3347,17 +3346,17 @@
       <c r="C59" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D59" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Nunca reenvia o link sozinha; status fica EM_ANALISE_AIVA (só o time muda)</t>
+          <t>Edu (AIVA) analisa o onboarding + CAF: aprova ou reprova</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr"/>
@@ -3382,11 +3381,11 @@
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Edu (AIVA) analisa o onboarding + CAF: aprova ou reprova</t>
+          <t>Aprovou → Nei move 50 → 70 (Treinar) · Reprovou → descarte</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr"/>
@@ -3411,11 +3410,11 @@
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Aprovou → Nei move 50 → 70 (Treinar) · Reprovou → descarte</t>
+          <t>Print do erro chega no chamado (📷) pro Nei identificar</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr"/>
@@ -3434,17 +3433,17 @@
       <c r="C62" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D62" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Print do erro chega no chamado (📷) pro Nei identificar</t>
+          <t>followup-fase 13h: 24h+ sem resposta → HSM 48 com miolo gerado pela Claude; máx 3 → escala Nei</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr"/>
@@ -3469,11 +3468,11 @@
         </is>
       </c>
       <c r="E63" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>followup-fase 13h: 24h+ sem resposta → HSM 48 com miolo gerado pela Claude; máx 3 → escala Nei</t>
+          <t>Respeita [PAUSA_ATE] e acionar_humano</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr"/>
@@ -3492,17 +3491,17 @@
       <c r="C64" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D64" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Respeita [PAUSA_ATE] e acionar_humano</t>
+          <t>Onboarding AIVA (retail-onboarding-hub) + CAF (biometria)</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr"/>
@@ -3527,11 +3526,11 @@
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>Onboarding AIVA (retail-onboarding-hub) + CAF (biometria)</t>
+          <t>sdr_chamados (erro relatado + print) → planilha Chamados</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr"/>
@@ -3540,27 +3539,27 @@
     </row>
     <row r="66">
       <c r="A66" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Em Análise AIVA</t>
+          <t>Treinar</t>
         </is>
       </c>
       <c r="C66" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D66" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>70</v>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>sdr_chamados (erro relatado + print) → planilha Chamados</t>
+          <t>Entrada na etapa → HSM 69 "Treinamento completo": link do Meet (seg/qui 9h30), Drive de materiais, cadastro de acessos</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr"/>
@@ -3585,11 +3584,11 @@
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → HSM 69 "Treinamento completo": link do Meet (seg/qui 9h30), Drive de materiais, cadastro de acessos</t>
+          <t>Regra de acessos (27/08): um usuário por loja; logins liberados pela AIVA após o treinamento</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr"/>
@@ -3614,11 +3613,11 @@
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Regra de acessos (27/08): um usuário por loja; logins liberados pela AIVA após o treinamento</t>
+          <t>Vacina da reprovação antes das primeiras consultas</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr"/>
@@ -3643,11 +3642,11 @@
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>Vacina da reprovação antes das primeiras consultas</t>
+          <t>🔒 Trava/desbloqueio de aparelho → só pelo Live Chat (Track não tem autoridade)</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr"/>
@@ -3672,11 +3671,11 @@
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>🔒 Trava/desbloqueio de aparelho → só pelo Live Chat (Track não tem autoridade)</t>
+          <t>Erro na tela → pede print → abre chamado pro Nei</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr"/>
@@ -3701,11 +3700,11 @@
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Erro na tela → pede print → abre chamado pro Nei</t>
+          <t>Loja nova no meio da conversa → aciona Nei (filial/correção cadastral)</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr"/>
@@ -3724,17 +3723,17 @@
       <c r="C72" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D72" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D72" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Loja nova no meio da conversa → aciona Nei (filial/correção cadastral)</t>
+          <t>Nei dá o treinamento (segundas e quintas, 9h30, mesmo link)</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr"/>
@@ -3759,11 +3758,11 @@
         </is>
       </c>
       <c r="E73" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Nei dá o treinamento (segundas e quintas, 9h30, mesmo link)</t>
+          <t>Nei confirma acesso/treino e move 70 → 71 (Login)</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr"/>
@@ -3782,17 +3781,17 @@
       <c r="C74" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D74" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D74" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>Nei confirma acesso/treino e move 70 → 71 (Login)</t>
+          <t>treinar-primeira-venda: disparo sob demanda (não é cron) — pergunta se já vendeu</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr"/>
@@ -3817,11 +3816,11 @@
         </is>
       </c>
       <c r="E75" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>treinar-primeira-venda: disparo sob demanda (não é cron) — pergunta se já vendeu</t>
+          <t>Lembretes de treinamento: scripts pontuais (ex.: aviso de feriado 04/09)</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr"/>
@@ -3840,17 +3839,17 @@
       <c r="C76" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D76" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D76" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Lembretes de treinamento: scripts pontuais (ex.: aviso de feriado 04/09)</t>
+          <t>Drive AIVA (materiais + vídeos Flexfone) · Google Meet</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr"/>
@@ -3875,11 +3874,11 @@
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Drive AIVA (materiais + vídeos Flexfone) · Google Meet</t>
+          <t>Apps Script "AIVA Docs" (linha/senha/atendimento manual)</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
@@ -3888,27 +3887,27 @@
     </row>
     <row r="78">
       <c r="A78" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Treinar</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C78" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="D78" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>71</v>
+      </c>
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Apps Script "AIVA Docs" (linha/senha/atendimento manual)</t>
+          <t>Espelha status LOGIN no painel (sync em tempo real)</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr"/>
@@ -3933,11 +3932,11 @@
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Espelha status LOGIN no painel (sync em tempo real)</t>
+          <t>Orienta primeiro acesso, operação Flexfone, consulta a distância × finalização presencial</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr"/>
@@ -3962,11 +3961,11 @@
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Orienta primeiro acesso, operação Flexfone, consulta a distância × finalização presencial</t>
+          <t>Boleto do cliente: quem emite é a LOJA, dentro do Flexfone — vídeo "Como emitir boleto"</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr"/>
@@ -3991,11 +3990,11 @@
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>Boleto do cliente: quem emite é a LOJA, dentro do Flexfone — vídeo "Como emitir boleto"</t>
+          <t>⛔ Regra 10/09: cliente novo = só AIVA no Flexfone; Odres congelada (segue só em lojas já abertas com ela)</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr"/>
@@ -4020,11 +4019,11 @@
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>⛔ Regra 10/09: cliente novo = só AIVA no Flexfone; Odres congelada (segue só em lojas já abertas com ela)</t>
+          <t>Links úteis por tema (portal, treinamento, 2ª via do cliente)</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr"/>
@@ -4043,17 +4042,17 @@
       <c r="C83" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D83" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D83" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>Links úteis por tema (portal, treinamento, 2ª via do cliente)</t>
+          <t>AIVA libera o login da loja</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr"/>
@@ -4078,11 +4077,11 @@
         </is>
       </c>
       <c r="E84" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>AIVA libera o login da loja</t>
+          <t>Nei acompanha a primeira venda e move 71 → 51</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr"/>
@@ -4101,17 +4100,17 @@
       <c r="C85" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D85" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D85" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>Nei acompanha a primeira venda e move 71 → 51</t>
+          <t>sla-liberacao: digest de lojas paradas em Treinar/Login — ⏸ desativado 06/08 (sob demanda)</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr"/>
@@ -4130,9 +4129,9 @@
       <c r="C86" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D86" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D86" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E86" s="4" t="n">
@@ -4140,7 +4139,7 @@
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>sla-liberacao: digest de lojas paradas em Treinar/Login — ⏸ desativado 06/08 (sob demanda)</t>
+          <t>Flexfone (plataforma da loja) · clientes.aivapay.com.br (2ª via)</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr"/>
@@ -4149,19 +4148,19 @@
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Loja Finalizada e Vendendo</t>
         </is>
       </c>
       <c r="C87" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="D87" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>51</v>
+      </c>
+      <c r="D87" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E87" s="4" t="n">
@@ -4169,7 +4168,7 @@
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Flexfone (plataforma da loja) · clientes.aivapay.com.br (2ª via)</t>
+          <t>Entrada na etapa → liga o relógio da consultoria ([CONSULTORIA_INICIO]) — não fala nada na hora</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr"/>
@@ -4194,11 +4193,11 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → liga o relógio da consultoria ([CONSULTORIA_INICIO]) — não fala nada na hora</t>
+          <t>FASE 5 — consultoria de vendas: playbook (preparar a loja · do CPF ao fechamento · aproveitar cada real · atrair fluxo)</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr"/>
@@ -4223,11 +4222,11 @@
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>FASE 5 — consultoria de vendas: playbook (preparar a loja · do CPF ao fechamento · aproveitar cada real · atrair fluxo)</t>
+          <t>Suporte pós-venda: A) lojista (plataforma/financeiro) · B) cliente final (parcelamento) · C) como fazer (Drive)</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr"/>
@@ -4252,11 +4251,11 @@
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Suporte pós-venda: A) lojista (plataforma/financeiro) · B) cliente final (parcelamento) · C) como fazer (Drive)</t>
+          <t>Objeção nº 1 "a AIVA não aprova" · prioriza autonomia do lojista</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr"/>
@@ -4281,11 +4280,11 @@
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Objeção nº 1 "a AIVA não aprova" · prioriza autonomia do lojista</t>
+          <t>Loja diz que nunca operou → 🚩 alerta Nei (loja_finalizada_sem_operar)</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr"/>
@@ -4310,11 +4309,11 @@
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Loja diz que nunca operou → 🚩 alerta Nei (loja_finalizada_sem_operar)</t>
+          <t>Repasse solicitado → planilha Repasses · CS acionamento → /atendimento</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr"/>
@@ -4333,17 +4332,17 @@
       <c r="C93" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D93" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Repasse solicitado → planilha Repasses · CS acionamento → /atendimento</t>
+          <t>Nei acompanha /desempenho (Portal Parceiros AIVA) e /atendimento (CS)</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr"/>
@@ -4368,11 +4367,11 @@
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Nei acompanha /desempenho (Portal Parceiros AIVA) e /atendimento (CS)</t>
+          <t>Comissão por loja ativada (importação mensal UME)</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr"/>
@@ -4397,11 +4396,11 @@
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>Comissão por loja ativada (importação mensal UME)</t>
+          <t>⚠️ Etapa 51 não aceita mover card pela API (só na mão)</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr"/>
@@ -4420,17 +4419,17 @@
       <c r="C96" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D96" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D96" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E96" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Etapa 51 não aceita mover card pela API (só na mão)</t>
+          <t>consultoria-vendas 14h seg–sex: D+7 e depois a cada 15d, 4 toques via HSM 48</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr"/>
@@ -4455,11 +4454,11 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>consultoria-vendas 14h seg–sex: D+7 e depois a cada 15d, 4 toques via HSM 48</t>
+          <t>check-primeira-venda terças 10h: loja quieta 7d+ → "a primeira venda saiu?" (máx 2, 30d)</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr"/>
@@ -4484,11 +4483,11 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>check-primeira-venda terças 10h: loja quieta 7d+ → "a primeira venda saiu?" (máx 2, 30d)</t>
+          <t>portal-aiva 6h todo dia: ativa loja (CNPJ registrado + Ativo no portal) + desempenho diário</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
@@ -4513,11 +4512,11 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>portal-aiva 6h todo dia: ativa loja (CNPJ registrado + Ativo no portal) + desempenho diário</t>
+          <t>pulso semanal segunda 8h30: fecha a semana e manda mensagens segmentadas às lojas ativas</t>
         </is>
       </c>
       <c r="G99" s="4" t="inlineStr"/>
@@ -4536,17 +4535,17 @@
       <c r="C100" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D100" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D100" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>pulso semanal segunda 8h30: fecha a semana e manda mensagens segmentadas às lojas ativas</t>
+          <t>Portal Parceiros AIVA → aiva_portal_diario (fonte) → aiva_desempenho (mês/semana)</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr"/>
@@ -4571,11 +4570,11 @@
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>Portal Parceiros AIVA → aiva_portal_diario (fonte) → aiva_desempenho (mês/semana)</t>
+          <t>sdr_repasses_solicitados → planilha Repasses · contas MRR no Evo</t>
         </is>
       </c>
       <c r="G101" s="4" t="inlineStr"/>
@@ -4584,27 +4583,27 @@
     </row>
     <row r="102">
       <c r="A102" s="4" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Loja Finalizada e Vendendo</t>
+          <t>Saídas do funil</t>
         </is>
       </c>
       <c r="C102" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="D102" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>53</v>
+      </c>
+      <c r="D102" s="22" t="inlineStr">
+        <is>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>sdr_repasses_solicitados → planilha Repasses · contas MRR no Evo</t>
+          <t>Interessado (Sem resposta) (automação 98): auto-descarte (Início +15d) · régua-saída · SEM_RESPOSTA +30d → DESCARTADO</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr"/>
@@ -4621,7 +4620,7 @@
         </is>
       </c>
       <c r="C103" s="4" t="n">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="D103" s="22" t="inlineStr">
         <is>
@@ -4629,11 +4628,11 @@
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Interessado (Sem resposta) (automação 98): auto-descarte (Início +15d) · régua-saída · SEM_RESPOSTA +30d → DESCARTADO</t>
+          <t>Bot Detectado (automação 100): VictorIA detectou auto-resposta; reativação recomeça do zero</t>
         </is>
       </c>
       <c r="G103" s="4" t="inlineStr"/>
@@ -4650,7 +4649,7 @@
         </is>
       </c>
       <c r="C104" s="4" t="n">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="D104" s="22" t="inlineStr">
         <is>
@@ -4658,11 +4657,11 @@
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Bot Detectado (automação 100): VictorIA detectou auto-resposta; reativação recomeça do zero</t>
+          <t>Lojas menos de 01 Ano (automação 101): CNPJ &lt; 1 ano na Receita → NAO_QUALIFICADO (regra 08/09)</t>
         </is>
       </c>
       <c r="G104" s="4" t="inlineStr"/>
@@ -4679,7 +4678,7 @@
         </is>
       </c>
       <c r="C105" s="4" t="n">
-        <v>93</v>
+        <v>19</v>
       </c>
       <c r="D105" s="22" t="inlineStr">
         <is>
@@ -4687,11 +4686,11 @@
         </is>
       </c>
       <c r="E105" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F105" s="4" t="inlineStr">
         <is>
-          <t>Lojas menos de 01 Ano (automação 101): CNPJ &lt; 1 ano na Receita → NAO_QUALIFICADO (regra 08/09)</t>
+          <t>Funil 19 · Odres / UME (transferência): CNPJ já na base AIVA/Odres → mensagem oficial + tag ODRES/UME · sdr_leads apaga o lead</t>
         </is>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
@@ -4707,20 +4706,18 @@
           <t>Saídas do funil</t>
         </is>
       </c>
-      <c r="C106" s="4" t="n">
-        <v>19</v>
-      </c>
+      <c r="C106" s="4" t="inlineStr"/>
       <c r="D106" s="22" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>Funil 19 · Odres / UME (transferência): CNPJ já na base AIVA/Odres → mensagem oficial + tag ODRES/UME · sdr_leads apaga o lead</t>
+          <t>OPT_OUT · LGPD (webhook): "não quero mais" → OPT_OUT · pedido de exclusão → confirma, apaga dados, guarda só o telefone</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr"/>
@@ -4743,11 +4740,11 @@
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F107" s="4" t="inlineStr">
         <is>
-          <t>OPT_OUT · LGPD (webhook): "não quero mais" → OPT_OUT · pedido de exclusão → confirma, apaga dados, guarda só o telefone</t>
+          <t>DESCARTADO / NAO_QUALIFICADO (terminal): Descarte manual do Nei é respeitado; status terminais nunca são revividos pelo sync</t>
         </is>
       </c>
       <c r="G107" s="4" t="inlineStr"/>
@@ -4756,25 +4753,25 @@
     </row>
     <row r="108">
       <c r="A108" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Saídas do funil</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr"/>
-      <c r="D108" s="22" t="inlineStr">
-        <is>
-          <t>Saída</t>
+      <c r="D108" s="23" t="inlineStr">
+        <is>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>DESCARTADO / NAO_QUALIFICADO (terminal): Descarte manual do Nei é respeitado; status terminais nunca são revividos pelo sync</t>
+          <t>🔁 Sincronização Evo ↔ painel: Cada etapa tem uma automação de entrada que chama /opportunity-stage (≈1 s). Reforço: sync-from-evo a cada 5 min, Evo é a fonte da verdade (exceções: descarte manual, terminais, guarda de 2 min).</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr"/>
@@ -4797,11 +4794,11 @@
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F109" s="4" t="inlineStr">
         <is>
-          <t>🔁 Sincronização Evo ↔ painel: Cada etapa tem uma automação de entrada que chama /opportunity-stage (≈1 s). Reforço: sync-from-evo a cada 5 min, Evo é a fonte da verdade (exceções: descarte manual, terminais, guarda de 2 min).</t>
+          <t>🛠 Auto-reprocess (10 min): Mensagem do lead sem resposta da VictorIA → reprocessa; falha da Claude → até N tentativas e depois escala humano.</t>
         </is>
       </c>
       <c r="G109" s="4" t="inlineStr"/>
@@ -4824,11 +4821,11 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>🛠 Auto-reprocess (10 min): Mensagem do lead sem resposta da VictorIA → reprocessa; falha da Claude → até N tentativas e depois escala humano.</t>
+          <t>👤 Fila humana: acionar_humano=true entra na fila: 🔴 ação · 📄 docs · 🟡 mover card. WhatsApp pro Nei 8h seg–sex + painel /atendimento (chamados, CS, travados, CNPJ).</t>
         </is>
       </c>
       <c r="G110" s="4" t="inlineStr"/>
@@ -4851,11 +4848,11 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>👤 Fila humana: acionar_humano=true entra na fila: 🔴 ação · 📄 docs · 🟡 mover card. WhatsApp pro Nei 8h seg–sex + painel /atendimento (chamados, CS, travados, CNPJ).</t>
+          <t>📋 Chamados: Erro relatado → pede print → sdr_chamados + planilha Chamados. Nei clica Resolver → planilha recebe "sim" e o chamado some.</t>
         </is>
       </c>
       <c r="G111" s="4" t="inlineStr"/>
@@ -4878,11 +4875,11 @@
         </is>
       </c>
       <c r="E112" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>📋 Chamados: Erro relatado → pede print → sdr_chamados + planilha Chamados. Nei clica Resolver → planilha recebe "sim" e o chamado some.</t>
+          <t>📣 Alertas: Transições de status alertam Nei/Aldo via WhatsApp (pré-aprovação, cadastro ✅, CAF confirmado, loja sem operar, contato a confirmar).</t>
         </is>
       </c>
       <c r="G112" s="4" t="inlineStr"/>
@@ -4905,11 +4902,11 @@
         </is>
       </c>
       <c r="E113" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F113" s="4" t="inlineStr">
         <is>
-          <t>📣 Alertas: Transições de status alertam Nei/Aldo via WhatsApp (pré-aprovação, cadastro ✅, CAF confirmado, loja sem operar, contato a confirmar).</t>
+          <t>📰 Briefings: briefing-pipeline 5h seg–sex (Aldo + Nei) · auditoria Evo × Supabase (só alerta) · destilador semanal sex 10h (curadoria).</t>
         </is>
       </c>
       <c r="G113" s="4" t="inlineStr"/>
@@ -4932,11 +4929,11 @@
         </is>
       </c>
       <c r="E114" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>📰 Briefings: briefing-pipeline 5h seg–sex (Aldo + Nei) · auditoria Evo × Supabase (só alerta) · destilador semanal sex 10h (curadoria).</t>
+          <t>🧠 VictorIA Analista: Widget do painel: consulta leads, conversas, chamados, repasses, desempenho semanal e curadoria. Só leitura.</t>
         </is>
       </c>
       <c r="G114" s="4" t="inlineStr"/>
@@ -4959,48 +4956,21 @@
         </is>
       </c>
       <c r="E115" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F115" s="4" t="inlineStr">
         <is>
-          <t>🧠 VictorIA Analista: Widget do painel: consulta leads, conversas, chamados, repasses, desempenho semanal e curadoria. Só leitura.</t>
+          <t>🗓 Data injetada a cada turno: A VictorIA não sabe o dia — lib/claude.ts injeta a data BRT fora do cache. Feriados/avisos entram como bloco dinâmico.</t>
         </is>
       </c>
       <c r="G115" s="4" t="inlineStr"/>
       <c r="H115" s="4" t="inlineStr"/>
       <c r="I115" s="4" t="inlineStr"/>
     </row>
-    <row r="116">
-      <c r="A116" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B116" s="4" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="C116" s="4" t="inlineStr"/>
-      <c r="D116" s="23" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="E116" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F116" s="4" t="inlineStr">
-        <is>
-          <t>🗓 Data injetada a cada turno: A VictorIA não sabe o dia — lib/claude.ts injeta a data BRT fora do cache. Feriados/avisos entram como bloco dinâmico.</t>
-        </is>
-      </c>
-      <c r="G116" s="4" t="inlineStr"/>
-      <c r="H116" s="4" t="inlineStr"/>
-      <c r="I116" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I116"/>
+  <autoFilter ref="A1:I115"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G116" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sim,não,mudar"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
chore(fluxo): remove nudge, reativacao, reengajamento e regua-saida da etapa Interessado (Aldo 10/09)
Limpeza pre-redesenho: as 4 rotinas saem do vercel.json e do codigo
(rotas apagadas; gerarReengajamento removida de lib/claude.ts). Fica so a
regua D+3/D+7/D+14 (/api/sdr/followup), PAUSADA ate o Aldo autorizar.

Lembrete de cobranca: linha fixa no briefing diario das 5h (Aldo + Nei)
em lib/pipeline-briefing.ts (+ bloco 'PENDENCIA ABERTA' no CLAUDE.md
local, que e gitignored). Apagar os dois no commit que religar a regua.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/fluxo-victoria-2026-09-10.xlsx
+++ b/docs/fluxo-victoria-2026-09-10.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etapas Evo" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Itens'!$A$1:$I$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Itens'!$A$1:$I$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Etapas Evo'!$A$1:$G$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -770,10 +770,10 @@
         <v>7</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J6" s="4" t="n">
         <v>3</v>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>auto-descarte (Início +15d) · régua-saída · SEM_RESPOSTA +30d → DESCARTADO</t>
+          <t>auto-descarte (Início +15d) · SEM_RESPOSTA +30d → DESCARTADO</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>• 53 · Interessado (Sem resposta) (automação 98): auto-descarte (Início +15d) · régua-saída · SEM_RESPOSTA +30d → DESCARTADO
+          <t>• 53 · Interessado (Sem resposta) (automação 98): auto-descarte (Início +15d) · SEM_RESPOSTA +30d → DESCARTADO
 • 69 · Bot Detectado (automação 100): VictorIA detectou auto-resposta; reativação recomeça do zero
 • 93 · Lojas menos de 01 Ano (automação 101): CNPJ &lt; 1 ano na Receita → NAO_QUALIFICADO (regra 08/09)
 • 19 · Funil 19 · Odres / UME (transferência): CNPJ já na base AIVA/Odres → mensagem oficial + tag ODRES/UME · sdr_leads apaga o lead
@@ -1409,7 +1409,7 @@
       </c>
       <c r="J3" s="13" t="inlineStr"/>
     </row>
-    <row r="4" ht="119" customHeight="1">
+    <row r="4" ht="111" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Humanos</t>
@@ -1423,8 +1423,7 @@
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
-          <t>• Nei entra quando: +10 lojas · pede contrato · irritado · dúvida técnica/jurídica · já cliente AIVA · confirmar_contato
-• Reengajamento esgotado (3×) → lead sinalizado; descartar é decisão do Nei</t>
+          <t>• Nei entra quando: +10 lojas · pede contrato · irritado · dúvida técnica/jurídica · já cliente AIVA · confirmar_contato</t>
         </is>
       </c>
       <c r="D4" s="13" t="inlineStr">
@@ -1468,7 +1467,7 @@
       </c>
       <c r="J4" s="13" t="inlineStr"/>
     </row>
-    <row r="5" ht="196" customHeight="1">
+    <row r="5" ht="197" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Rotinas automáticas</t>
@@ -1477,17 +1476,14 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>• HSM 41 "AIVA Dia 1" (D+0) → lead INICIO + card 66
-• Régua D+3 (HSM 35) · D+7 (HSM 38) · D+14 (HSM 39) — ⏸ PAUSADA (17/08; religada e pausada de novo em 10/09): ~4.100 leads vencidos aguardam o fluxo novo
+• Régua D+3 (HSM 35) · D+7 (HSM 38) · D+14 (HSM 39) — ⏸ PAUSADA até o Aldo autorizar (única cadência que fica): ~4.100 leads vencidos aguardam o fluxo novo
 • auto-descarte 10h seg–sex: INICIO +15d sem resposta → card 53 + SEM_RESPOSTA
 • varredura de lojas 10h (todo dia) → Excel parcial + fila_disparo (4.777 na fila)</t>
         </is>
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>• nudge 12h (Vercel): conversa parada 3–24h → cutucada contextual (máx 2)
-• reativação 10h: parado 48h–14d → HSM 48 (20/execução)
-• reengajamento 16h seg–sex: follow-up personalizado via HSM 48, até 3× a cada 15d
-• régua-saída 10h30: 3 reengajamentos + 15d mudo + bola com o lead → card 53 + SEM_RESPOSTA
+          <t>• Nenhuma cutucada automática (nudge, reativação, reengajamento e régua-saída removidos em 10/09)
 • auto-descarte: INTERESSADO +21d sem msg do lead → AGUARDANDO</t>
         </is>
       </c>
@@ -1620,7 +1616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1964,7 +1960,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Régua D+3 (HSM 35) · D+7 (HSM 38) · D+14 (HSM 39) — ⏸ PAUSADA (17/08; religada e pausada de novo em 10/09): ~4.100 leads vencidos aguardam o fluxo novo</t>
+          <t>Régua D+3 (HSM 35) · D+7 (HSM 38) · D+14 (HSM 39) — ⏸ PAUSADA até o Aldo autorizar (única cadência que fica): ~4.100 leads vencidos aguardam o fluxo novo</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr"/>
@@ -2331,17 +2327,17 @@
       <c r="C24" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Reengajamento esgotado (3×) → lead sinalizado; descartar é decisão do Nei</t>
+          <t>Nenhuma cutucada automática (nudge, reativação, reengajamento e régua-saída removidos em 10/09)</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr"/>
@@ -2366,11 +2362,11 @@
         </is>
       </c>
       <c r="E25" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>nudge 12h (Vercel): conversa parada 3–24h → cutucada contextual (máx 2)</t>
+          <t>auto-descarte: INTERESSADO +21d sem msg do lead → AGUARDANDO</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr"/>
@@ -2389,17 +2385,17 @@
       <c r="C26" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="D26" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E26" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>reativação 10h: parado 48h–14d → HSM 48 (20/execução)</t>
+          <t>BrasilAPI (Receita): idade, situação, QSA — marcador [CNPJ_RECEITA] impede revalidar</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr"/>
@@ -2418,17 +2414,17 @@
       <c r="C27" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D27" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E27" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>reengajamento 16h seg–sex: follow-up personalizado via HSM 48, até 3× a cada 15d</t>
+          <t>aiva_base_cnpjs (6.323 CNPJs, importada 11h todo dia via Data Studio)</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr"/>
@@ -2447,17 +2443,17 @@
       <c r="C28" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="D28" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>régua-saída 10h30: 3 reengajamentos + 15d mudo + bola com o lead → card 53 + SEM_RESPOSTA</t>
+          <t>sdr_registros_cnpj (status informada) · formsdata da opp no Evo</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr"/>
@@ -2466,27 +2462,27 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Interessado</t>
+          <t>Pré Aprovação</t>
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>54</v>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>auto-descarte: INTERESSADO +21d sem msg do lead → AGUARDANDO</t>
+          <t>FASE 2 — só tranquiliza: "estamos analisando, em breve retorno". Não pede dado, não promete prazo</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr"/>
@@ -2495,27 +2491,27 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Interessado</t>
+          <t>Pré Aprovação</t>
         </is>
       </c>
       <c r="C30" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="D30" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>54</v>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>BrasilAPI (Receita): idade, situação, QSA — marcador [CNPJ_RECEITA] impede revalidar</t>
+          <t>Se o CNPJ tiver ≥ 3 lojas → tag IMPORTANTE (74) na opp</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr"/>
@@ -2524,27 +2520,27 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Interessado</t>
+          <t>Pré Aprovação</t>
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="D31" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>54</v>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>aiva_base_cnpjs (6.323 CNPJs, importada 11h todo dia via Data Studio)</t>
+          <t>Alerta Nei + Aldo: pré-aprovação enviada</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr"/>
@@ -2553,27 +2549,27 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Interessado</t>
+          <t>Pré Aprovação</t>
         </is>
       </c>
       <c r="C32" s="4" t="n">
-        <v>47</v>
-      </c>
-      <c r="D32" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>54</v>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>sdr_registros_cnpj (status informada) · formsdata da opp no Evo</t>
+          <t>Edu (AIVA) analisa a pré-aprovação pela planilha, em até 24h</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr"/>
@@ -2592,17 +2588,17 @@
       <c r="C33" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D33" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>FASE 2 — só tranquiliza: "estamos analisando, em breve retorno". Não pede dado, não promete prazo</t>
+          <t>Aprovou → Nei move o card 54 → 49 (Cadastro Recebido)</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr"/>
@@ -2621,17 +2617,17 @@
       <c r="C34" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D34" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Se o CNPJ tiver ≥ 3 lojas → tag IMPORTANTE (74) na opp</t>
+          <t>Reprovou → descarte (Nei marca no Evo)</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr"/>
@@ -2650,17 +2646,17 @@
       <c r="C35" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D35" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D35" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Alerta Nei + Aldo: pré-aprovação enviada</t>
+          <t>Nenhuma cobrança automática nessa etapa (espera humana)</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr"/>
@@ -2679,9 +2675,9 @@
       <c r="C36" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
@@ -2689,7 +2685,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Edu (AIVA) analisa a pré-aprovação pela planilha, em até 24h</t>
+          <t>Planilha AIVA APROVAÇÃO (Google Sheets) — linha por lead pré-aprovado</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr"/>
@@ -2708,9 +2704,9 @@
       <c r="C37" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
@@ -2718,7 +2714,7 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Aprovou → Nei move o card 54 → 49 (Cadastro Recebido)</t>
+          <t>Tags Evo: AIVA (69) sempre · IMPORTANTE (74) se ≥ 3 lojas</t>
         </is>
       </c>
       <c r="G37" s="4" t="inlineStr"/>
@@ -2727,27 +2723,27 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Pré Aprovação</t>
+          <t>Cadastro Recebido</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+        <v>49</v>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Reprovou → descarte (Nei marca no Evo)</t>
+          <t>Entrada na etapa → HSM 29 "Complete o cadastro" reabre a janela; status volta a INTERESSADO com marcador de Fase 3</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr"/>
@@ -2756,27 +2752,27 @@
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Pré Aprovação</t>
+          <t>Cadastro Recebido</t>
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="D39" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>49</v>
+      </c>
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Nenhuma cobrança automática nessa etapa (espera humana)</t>
+          <t>FASE 3 — coleta 5 dados: e-mail do sócio · faturamento anual · boleto mensal · localização das lojas · CNPJs adicionais (só se ≥ 2 lojas)</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr"/>
@@ -2785,27 +2781,27 @@
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Cadastro Recebido</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="D40" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Pré Aprovação</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="D40" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Planilha AIVA APROVAÇÃO (Google Sheets) — linha por lead pré-aprovado</t>
+          <t>Dados sensíveis: explica o porquê, aceita "por alto"; recusa → aciona humano (receio_dados_sensiveis)</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr"/>
@@ -2814,27 +2810,27 @@
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Pré Aprovação</t>
+          <t>Cadastro Recebido</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
-        <v>54</v>
-      </c>
-      <c r="D41" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>49</v>
+      </c>
+      <c r="D41" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Tags Evo: AIVA (69) sempre · IMPORTANTE (74) se ≥ 3 lojas</t>
+          <t>Trava anti-conclusão: sem os 5, nunca diz "cadastro completo"</t>
         </is>
       </c>
       <c r="G41" s="4" t="inlineStr"/>
@@ -2859,11 +2855,11 @@
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → HSM 29 "Complete o cadastro" reabre a janela; status volta a INTERESSADO com marcador de Fase 3</t>
+          <t>12 dados completos → CADASTRO_RECEBIDO + HubSpot + registro do CNPJ + alerta ✅ (cadastro_completo)</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr"/>
@@ -2882,17 +2878,17 @@
       <c r="C43" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D43" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D43" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>FASE 3 — coleta 5 dados: e-mail do sócio · faturamento anual · boleto mensal · localização das lojas · CNPJs adicionais (só se ≥ 2 lojas)</t>
+          <t>Nei confere no /registros e move o card 49 → 50 (Em Análise)</t>
         </is>
       </c>
       <c r="G43" s="4" t="inlineStr"/>
@@ -2911,17 +2907,17 @@
       <c r="C44" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D44" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D44" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Dados sensíveis: explica o porquê, aceita "por alto"; recusa → aciona humano (receio_dados_sensiveis)</t>
+          <t>Cobrança esgotada (3 toques) → escala pro Nei uma vez</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr"/>
@@ -2940,17 +2936,17 @@
       <c r="C45" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D45" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D45" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Trava anti-conclusão: sem os 5, nunca diz "cadastro completo"</t>
+          <t>cadastro-recebido-cobranca 15h seg–sex: D+1 · D+3 · D+7 na etapa → HSM 48 + pede o dado que falta (um por vez)</t>
         </is>
       </c>
       <c r="G45" s="4" t="inlineStr"/>
@@ -2969,17 +2965,17 @@
       <c r="C46" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D46" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D46" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E46" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>12 dados completos → CADASTRO_RECEBIDO + HubSpot + registro do CNPJ + alerta ✅ (cadastro_completo)</t>
+          <t>Fonte da verdade = etapa do Evo (stagebegintime)</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr"/>
@@ -2998,9 +2994,9 @@
       <c r="C47" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D47" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D47" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E47" s="4" t="n">
@@ -3008,7 +3004,7 @@
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Nei confere no /registros e move o card 49 → 50 (Em Análise)</t>
+          <t>HubSpot (contato/empresa) — só quando os 12 dados fecham</t>
         </is>
       </c>
       <c r="G47" s="4" t="inlineStr"/>
@@ -3027,9 +3023,9 @@
       <c r="C48" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D48" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D48" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E48" s="4" t="n">
@@ -3037,7 +3033,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Cobrança esgotada (3 toques) → escala pro Nei uma vez</t>
+          <t>sdr_registros_cnpj (matriz + adicionais) · formsdata da opp</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr"/>
@@ -3056,17 +3052,17 @@
       <c r="C49" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="D49" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D49" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E49" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>cadastro-recebido-cobranca 15h seg–sex: D+1 · D+3 · D+7 na etapa → HSM 48 + pede o dado que falta (um por vez)</t>
+          <t>Painel /registros</t>
         </is>
       </c>
       <c r="G49" s="4" t="inlineStr"/>
@@ -3075,27 +3071,27 @@
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Cadastro Recebido</t>
+          <t>Em Análise AIVA</t>
         </is>
       </c>
       <c r="C50" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="D50" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>50</v>
+      </c>
+      <c r="D50" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E50" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Fonte da verdade = etapa do Evo (stagebegintime)</t>
+          <t>Entrada na etapa → HSM 34 (aprovação) com o link do onboarding retail-onboarding-hub + biometria (CAF)</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr"/>
@@ -3104,27 +3100,27 @@
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Cadastro Recebido</t>
+          <t>Em Análise AIVA</t>
         </is>
       </c>
       <c r="C51" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="D51" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>50</v>
+      </c>
+      <c r="D51" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>HubSpot (contato/empresa) — só quando os 12 dados fecham</t>
+          <t>FASE 4 — acompanha: "conseguiu acessar? concluiu a biometria?"</t>
         </is>
       </c>
       <c r="G51" s="4" t="inlineStr"/>
@@ -3133,27 +3129,27 @@
     </row>
     <row r="52">
       <c r="A52" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Cadastro Recebido</t>
+          <t>Em Análise AIVA</t>
         </is>
       </c>
       <c r="C52" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="D52" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>50</v>
+      </c>
+      <c r="D52" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E52" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>sdr_registros_cnpj (matriz + adicionais) · formsdata da opp</t>
+          <t>Qualquer erro → PEDE O PRINT primeiro (regra 08/09) · dificuldade → aciona humano (dificuldade_onboarding_caf)</t>
         </is>
       </c>
       <c r="G52" s="4" t="inlineStr"/>
@@ -3162,27 +3158,27 @@
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Em Análise AIVA</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>Cadastro Recebido</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="n">
-        <v>49</v>
-      </c>
-      <c r="D53" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="n">
-        <v>3</v>
-      </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Painel /registros</t>
+          <t>Lead diz que concluiu → aciona humano (cadastro_caf_confirmado)</t>
         </is>
       </c>
       <c r="G53" s="4" t="inlineStr"/>
@@ -3207,11 +3203,11 @@
         </is>
       </c>
       <c r="E54" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → HSM 34 (aprovação) com o link do onboarding retail-onboarding-hub + biometria (CAF)</t>
+          <t>Nunca reenvia o link sozinha; status fica EM_ANALISE_AIVA (só o time muda)</t>
         </is>
       </c>
       <c r="G54" s="4" t="inlineStr"/>
@@ -3230,17 +3226,17 @@
       <c r="C55" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D55" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E55" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>FASE 4 — acompanha: "conseguiu acessar? concluiu a biometria?"</t>
+          <t>Edu (AIVA) analisa o onboarding + CAF: aprova ou reprova</t>
         </is>
       </c>
       <c r="G55" s="4" t="inlineStr"/>
@@ -3259,17 +3255,17 @@
       <c r="C56" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D56" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E56" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Qualquer erro → PEDE O PRINT primeiro (regra 08/09) · dificuldade → aciona humano (dificuldade_onboarding_caf)</t>
+          <t>Aprovou → Nei move 50 → 70 (Treinar) · Reprovou → descarte</t>
         </is>
       </c>
       <c r="G56" s="4" t="inlineStr"/>
@@ -3288,17 +3284,17 @@
       <c r="C57" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D57" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E57" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F57" s="4" t="inlineStr">
         <is>
-          <t>Lead diz que concluiu → aciona humano (cadastro_caf_confirmado)</t>
+          <t>Print do erro chega no chamado (📷) pro Nei identificar</t>
         </is>
       </c>
       <c r="G57" s="4" t="inlineStr"/>
@@ -3317,17 +3313,17 @@
       <c r="C58" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D58" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E58" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Nunca reenvia o link sozinha; status fica EM_ANALISE_AIVA (só o time muda)</t>
+          <t>followup-fase 13h: 24h+ sem resposta → HSM 48 com miolo gerado pela Claude; máx 3 → escala Nei</t>
         </is>
       </c>
       <c r="G58" s="4" t="inlineStr"/>
@@ -3346,17 +3342,17 @@
       <c r="C59" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D59" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E59" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" s="4" t="inlineStr">
         <is>
-          <t>Edu (AIVA) analisa o onboarding + CAF: aprova ou reprova</t>
+          <t>Respeita [PAUSA_ATE] e acionar_humano</t>
         </is>
       </c>
       <c r="G59" s="4" t="inlineStr"/>
@@ -3375,17 +3371,17 @@
       <c r="C60" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E60" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>Aprovou → Nei move 50 → 70 (Treinar) · Reprovou → descarte</t>
+          <t>Onboarding AIVA (retail-onboarding-hub) + CAF (biometria)</t>
         </is>
       </c>
       <c r="G60" s="4" t="inlineStr"/>
@@ -3404,17 +3400,17 @@
       <c r="C61" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D61" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E61" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>Print do erro chega no chamado (📷) pro Nei identificar</t>
+          <t>sdr_chamados (erro relatado + print) → planilha Chamados</t>
         </is>
       </c>
       <c r="G61" s="4" t="inlineStr"/>
@@ -3423,19 +3419,19 @@
     </row>
     <row r="62">
       <c r="A62" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Em Análise AIVA</t>
+          <t>Treinar</t>
         </is>
       </c>
       <c r="C62" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D62" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>70</v>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E62" s="4" t="n">
@@ -3443,7 +3439,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>followup-fase 13h: 24h+ sem resposta → HSM 48 com miolo gerado pela Claude; máx 3 → escala Nei</t>
+          <t>Entrada na etapa → HSM 69 "Treinamento completo": link do Meet (seg/qui 9h30), Drive de materiais, cadastro de acessos</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr"/>
@@ -3452,19 +3448,19 @@
     </row>
     <row r="63">
       <c r="A63" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Em Análise AIVA</t>
+          <t>Treinar</t>
         </is>
       </c>
       <c r="C63" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D63" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>70</v>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E63" s="4" t="n">
@@ -3472,7 +3468,7 @@
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Respeita [PAUSA_ATE] e acionar_humano</t>
+          <t>Regra de acessos (27/08): um usuário por loja; logins liberados pela AIVA após o treinamento</t>
         </is>
       </c>
       <c r="G63" s="4" t="inlineStr"/>
@@ -3481,27 +3477,27 @@
     </row>
     <row r="64">
       <c r="A64" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Em Análise AIVA</t>
+          <t>Treinar</t>
         </is>
       </c>
       <c r="C64" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D64" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>70</v>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E64" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>Onboarding AIVA (retail-onboarding-hub) + CAF (biometria)</t>
+          <t>Vacina da reprovação antes das primeiras consultas</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr"/>
@@ -3510,27 +3506,27 @@
     </row>
     <row r="65">
       <c r="A65" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Em Análise AIVA</t>
+          <t>Treinar</t>
         </is>
       </c>
       <c r="C65" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D65" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>70</v>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E65" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F65" s="4" t="inlineStr">
         <is>
-          <t>sdr_chamados (erro relatado + print) → planilha Chamados</t>
+          <t>🔒 Trava/desbloqueio de aparelho → só pelo Live Chat (Track não tem autoridade)</t>
         </is>
       </c>
       <c r="G65" s="4" t="inlineStr"/>
@@ -3555,11 +3551,11 @@
         </is>
       </c>
       <c r="E66" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → HSM 69 "Treinamento completo": link do Meet (seg/qui 9h30), Drive de materiais, cadastro de acessos</t>
+          <t>Erro na tela → pede print → abre chamado pro Nei</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr"/>
@@ -3584,11 +3580,11 @@
         </is>
       </c>
       <c r="E67" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>Regra de acessos (27/08): um usuário por loja; logins liberados pela AIVA após o treinamento</t>
+          <t>Loja nova no meio da conversa → aciona Nei (filial/correção cadastral)</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr"/>
@@ -3607,17 +3603,17 @@
       <c r="C68" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D68" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D68" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E68" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Vacina da reprovação antes das primeiras consultas</t>
+          <t>Nei dá o treinamento (segundas e quintas, 9h30, mesmo link)</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr"/>
@@ -3636,17 +3632,17 @@
       <c r="C69" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D69" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D69" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E69" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F69" s="4" t="inlineStr">
         <is>
-          <t>🔒 Trava/desbloqueio de aparelho → só pelo Live Chat (Track não tem autoridade)</t>
+          <t>Nei confirma acesso/treino e move 70 → 71 (Login)</t>
         </is>
       </c>
       <c r="G69" s="4" t="inlineStr"/>
@@ -3665,17 +3661,17 @@
       <c r="C70" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D70" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D70" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E70" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Erro na tela → pede print → abre chamado pro Nei</t>
+          <t>treinar-primeira-venda: disparo sob demanda (não é cron) — pergunta se já vendeu</t>
         </is>
       </c>
       <c r="G70" s="4" t="inlineStr"/>
@@ -3694,17 +3690,17 @@
       <c r="C71" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D71" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D71" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E71" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Loja nova no meio da conversa → aciona Nei (filial/correção cadastral)</t>
+          <t>Lembretes de treinamento: scripts pontuais (ex.: aviso de feriado 04/09)</t>
         </is>
       </c>
       <c r="G71" s="4" t="inlineStr"/>
@@ -3723,9 +3719,9 @@
       <c r="C72" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D72" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E72" s="4" t="n">
@@ -3733,7 +3729,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Nei dá o treinamento (segundas e quintas, 9h30, mesmo link)</t>
+          <t>Drive AIVA (materiais + vídeos Flexfone) · Google Meet</t>
         </is>
       </c>
       <c r="G72" s="4" t="inlineStr"/>
@@ -3752,9 +3748,9 @@
       <c r="C73" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="D73" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D73" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E73" s="4" t="n">
@@ -3762,7 +3758,7 @@
       </c>
       <c r="F73" s="4" t="inlineStr">
         <is>
-          <t>Nei confirma acesso/treino e move 70 → 71 (Login)</t>
+          <t>Apps Script "AIVA Docs" (linha/senha/atendimento manual)</t>
         </is>
       </c>
       <c r="G73" s="4" t="inlineStr"/>
@@ -3771,19 +3767,19 @@
     </row>
     <row r="74">
       <c r="A74" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Treinar</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C74" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="D74" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>71</v>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E74" s="4" t="n">
@@ -3791,7 +3787,7 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>treinar-primeira-venda: disparo sob demanda (não é cron) — pergunta se já vendeu</t>
+          <t>Espelha status LOGIN no painel (sync em tempo real)</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr"/>
@@ -3800,19 +3796,19 @@
     </row>
     <row r="75">
       <c r="A75" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Treinar</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C75" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="D75" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>71</v>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E75" s="4" t="n">
@@ -3820,7 +3816,7 @@
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>Lembretes de treinamento: scripts pontuais (ex.: aviso de feriado 04/09)</t>
+          <t>Orienta primeiro acesso, operação Flexfone, consulta a distância × finalização presencial</t>
         </is>
       </c>
       <c r="G75" s="4" t="inlineStr"/>
@@ -3829,27 +3825,27 @@
     </row>
     <row r="76">
       <c r="A76" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Treinar</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C76" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="D76" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>71</v>
+      </c>
+      <c r="D76" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E76" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>Drive AIVA (materiais + vídeos Flexfone) · Google Meet</t>
+          <t>Boleto do cliente: quem emite é a LOJA, dentro do Flexfone — vídeo "Como emitir boleto"</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr"/>
@@ -3858,27 +3854,27 @@
     </row>
     <row r="77">
       <c r="A77" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Treinar</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="C77" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="D77" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>71</v>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E77" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>Apps Script "AIVA Docs" (linha/senha/atendimento manual)</t>
+          <t>⛔ Regra 10/09: cliente novo = só AIVA no Flexfone; Odres congelada (segue só em lojas já abertas com ela)</t>
         </is>
       </c>
       <c r="G77" s="4" t="inlineStr"/>
@@ -3903,11 +3899,11 @@
         </is>
       </c>
       <c r="E78" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>Espelha status LOGIN no painel (sync em tempo real)</t>
+          <t>Links úteis por tema (portal, treinamento, 2ª via do cliente)</t>
         </is>
       </c>
       <c r="G78" s="4" t="inlineStr"/>
@@ -3926,17 +3922,17 @@
       <c r="C79" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D79" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D79" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E79" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F79" s="4" t="inlineStr">
         <is>
-          <t>Orienta primeiro acesso, operação Flexfone, consulta a distância × finalização presencial</t>
+          <t>AIVA libera o login da loja</t>
         </is>
       </c>
       <c r="G79" s="4" t="inlineStr"/>
@@ -3955,17 +3951,17 @@
       <c r="C80" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D80" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D80" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E80" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>Boleto do cliente: quem emite é a LOJA, dentro do Flexfone — vídeo "Como emitir boleto"</t>
+          <t>Nei acompanha a primeira venda e move 71 → 51</t>
         </is>
       </c>
       <c r="G80" s="4" t="inlineStr"/>
@@ -3984,17 +3980,17 @@
       <c r="C81" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D81" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D81" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E81" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>⛔ Regra 10/09: cliente novo = só AIVA no Flexfone; Odres congelada (segue só em lojas já abertas com ela)</t>
+          <t>sla-liberacao: digest de lojas paradas em Treinar/Login — ⏸ desativado 06/08 (sob demanda)</t>
         </is>
       </c>
       <c r="G81" s="4" t="inlineStr"/>
@@ -4013,17 +4009,17 @@
       <c r="C82" s="4" t="n">
         <v>71</v>
       </c>
-      <c r="D82" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D82" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E82" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>Links úteis por tema (portal, treinamento, 2ª via do cliente)</t>
+          <t>Flexfone (plataforma da loja) · clientes.aivapay.com.br (2ª via)</t>
         </is>
       </c>
       <c r="G82" s="4" t="inlineStr"/>
@@ -4032,19 +4028,19 @@
     </row>
     <row r="83">
       <c r="A83" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Loja Finalizada e Vendendo</t>
         </is>
       </c>
       <c r="C83" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="D83" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+        <v>51</v>
+      </c>
+      <c r="D83" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E83" s="4" t="n">
@@ -4052,7 +4048,7 @@
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>AIVA libera o login da loja</t>
+          <t>Entrada na etapa → liga o relógio da consultoria ([CONSULTORIA_INICIO]) — não fala nada na hora</t>
         </is>
       </c>
       <c r="G83" s="4" t="inlineStr"/>
@@ -4061,19 +4057,19 @@
     </row>
     <row r="84">
       <c r="A84" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Loja Finalizada e Vendendo</t>
         </is>
       </c>
       <c r="C84" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="D84" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+        <v>51</v>
+      </c>
+      <c r="D84" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E84" s="4" t="n">
@@ -4081,7 +4077,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>Nei acompanha a primeira venda e move 71 → 51</t>
+          <t>FASE 5 — consultoria de vendas: playbook (preparar a loja · do CPF ao fechamento · aproveitar cada real · atrair fluxo)</t>
         </is>
       </c>
       <c r="G84" s="4" t="inlineStr"/>
@@ -4090,27 +4086,27 @@
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Loja Finalizada e Vendendo</t>
         </is>
       </c>
       <c r="C85" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="D85" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>51</v>
+      </c>
+      <c r="D85" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E85" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>sla-liberacao: digest de lojas paradas em Treinar/Login — ⏸ desativado 06/08 (sob demanda)</t>
+          <t>Suporte pós-venda: A) lojista (plataforma/financeiro) · B) cliente final (parcelamento) · C) como fazer (Drive)</t>
         </is>
       </c>
       <c r="G85" s="4" t="inlineStr"/>
@@ -4119,27 +4115,27 @@
     </row>
     <row r="86">
       <c r="A86" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Loja Finalizada e Vendendo</t>
         </is>
       </c>
       <c r="C86" s="4" t="n">
-        <v>71</v>
-      </c>
-      <c r="D86" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>51</v>
+      </c>
+      <c r="D86" s="18" t="inlineStr">
+        <is>
+          <t>VictorIA</t>
         </is>
       </c>
       <c r="E86" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>Flexfone (plataforma da loja) · clientes.aivapay.com.br (2ª via)</t>
+          <t>Objeção nº 1 "a AIVA não aprova" · prioriza autonomia do lojista</t>
         </is>
       </c>
       <c r="G86" s="4" t="inlineStr"/>
@@ -4164,11 +4160,11 @@
         </is>
       </c>
       <c r="E87" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F87" s="4" t="inlineStr">
         <is>
-          <t>Entrada na etapa → liga o relógio da consultoria ([CONSULTORIA_INICIO]) — não fala nada na hora</t>
+          <t>Loja diz que nunca operou → 🚩 alerta Nei (loja_finalizada_sem_operar)</t>
         </is>
       </c>
       <c r="G87" s="4" t="inlineStr"/>
@@ -4193,11 +4189,11 @@
         </is>
       </c>
       <c r="E88" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>FASE 5 — consultoria de vendas: playbook (preparar a loja · do CPF ao fechamento · aproveitar cada real · atrair fluxo)</t>
+          <t>Repasse solicitado → planilha Repasses · CS acionamento → /atendimento</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr"/>
@@ -4216,17 +4212,17 @@
       <c r="C89" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D89" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D89" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E89" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F89" s="4" t="inlineStr">
         <is>
-          <t>Suporte pós-venda: A) lojista (plataforma/financeiro) · B) cliente final (parcelamento) · C) como fazer (Drive)</t>
+          <t>Nei acompanha /desempenho (Portal Parceiros AIVA) e /atendimento (CS)</t>
         </is>
       </c>
       <c r="G89" s="4" t="inlineStr"/>
@@ -4245,17 +4241,17 @@
       <c r="C90" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D90" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E90" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>Objeção nº 1 "a AIVA não aprova" · prioriza autonomia do lojista</t>
+          <t>Comissão por loja ativada (importação mensal UME)</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr"/>
@@ -4274,17 +4270,17 @@
       <c r="C91" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D91" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D91" s="19" t="inlineStr">
+        <is>
+          <t>Humanos</t>
         </is>
       </c>
       <c r="E91" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F91" s="4" t="inlineStr">
         <is>
-          <t>Loja diz que nunca operou → 🚩 alerta Nei (loja_finalizada_sem_operar)</t>
+          <t>⚠️ Etapa 51 não aceita mover card pela API (só na mão)</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr"/>
@@ -4303,17 +4299,17 @@
       <c r="C92" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D92" s="18" t="inlineStr">
-        <is>
-          <t>VictorIA</t>
+      <c r="D92" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E92" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Repasse solicitado → planilha Repasses · CS acionamento → /atendimento</t>
+          <t>consultoria-vendas 14h seg–sex: D+7 e depois a cada 15d, 4 toques via HSM 48</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr"/>
@@ -4332,17 +4328,17 @@
       <c r="C93" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D93" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D93" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E93" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F93" s="4" t="inlineStr">
         <is>
-          <t>Nei acompanha /desempenho (Portal Parceiros AIVA) e /atendimento (CS)</t>
+          <t>check-primeira-venda terças 10h: loja quieta 7d+ → "a primeira venda saiu?" (máx 2, 30d)</t>
         </is>
       </c>
       <c r="G93" s="4" t="inlineStr"/>
@@ -4361,17 +4357,17 @@
       <c r="C94" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D94" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D94" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E94" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>Comissão por loja ativada (importação mensal UME)</t>
+          <t>portal-aiva 6h todo dia: ativa loja (CNPJ registrado + Ativo no portal) + desempenho diário</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr"/>
@@ -4390,17 +4386,17 @@
       <c r="C95" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D95" s="19" t="inlineStr">
-        <is>
-          <t>Humanos</t>
+      <c r="D95" s="20" t="inlineStr">
+        <is>
+          <t>Rotinas automáticas</t>
         </is>
       </c>
       <c r="E95" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F95" s="4" t="inlineStr">
         <is>
-          <t>⚠️ Etapa 51 não aceita mover card pela API (só na mão)</t>
+          <t>pulso semanal segunda 8h30: fecha a semana e manda mensagens segmentadas às lojas ativas</t>
         </is>
       </c>
       <c r="G95" s="4" t="inlineStr"/>
@@ -4419,9 +4415,9 @@
       <c r="C96" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D96" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D96" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E96" s="4" t="n">
@@ -4429,7 +4425,7 @@
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>consultoria-vendas 14h seg–sex: D+7 e depois a cada 15d, 4 toques via HSM 48</t>
+          <t>Portal Parceiros AIVA → aiva_portal_diario (fonte) → aiva_desempenho (mês/semana)</t>
         </is>
       </c>
       <c r="G96" s="4" t="inlineStr"/>
@@ -4448,9 +4444,9 @@
       <c r="C97" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="D97" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+      <c r="D97" s="21" t="inlineStr">
+        <is>
+          <t>Sistemas e dados</t>
         </is>
       </c>
       <c r="E97" s="4" t="n">
@@ -4458,7 +4454,7 @@
       </c>
       <c r="F97" s="4" t="inlineStr">
         <is>
-          <t>check-primeira-venda terças 10h: loja quieta 7d+ → "a primeira venda saiu?" (máx 2, 30d)</t>
+          <t>sdr_repasses_solicitados → planilha Repasses · contas MRR no Evo</t>
         </is>
       </c>
       <c r="G97" s="4" t="inlineStr"/>
@@ -4467,27 +4463,27 @@
     </row>
     <row r="98">
       <c r="A98" s="4" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Loja Finalizada e Vendendo</t>
+          <t>Saídas do funil</t>
         </is>
       </c>
       <c r="C98" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="D98" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>53</v>
+      </c>
+      <c r="D98" s="22" t="inlineStr">
+        <is>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>portal-aiva 6h todo dia: ativa loja (CNPJ registrado + Ativo no portal) + desempenho diário</t>
+          <t>Interessado (Sem resposta) (automação 98): auto-descarte (Início +15d) · SEM_RESPOSTA +30d → DESCARTADO</t>
         </is>
       </c>
       <c r="G98" s="4" t="inlineStr"/>
@@ -4496,27 +4492,27 @@
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Loja Finalizada e Vendendo</t>
+          <t>Saídas do funil</t>
         </is>
       </c>
       <c r="C99" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="D99" s="20" t="inlineStr">
-        <is>
-          <t>Rotinas automáticas</t>
+        <v>69</v>
+      </c>
+      <c r="D99" s="22" t="inlineStr">
+        <is>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>pulso semanal segunda 8h30: fecha a semana e manda mensagens segmentadas às lojas ativas</t>
+          <t>Bot Detectado (automação 100): VictorIA detectou auto-resposta; reativação recomeça do zero</t>
         </is>
       </c>
       <c r="G99" s="4" t="inlineStr"/>
@@ -4525,27 +4521,27 @@
     </row>
     <row r="100">
       <c r="A100" s="4" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Loja Finalizada e Vendendo</t>
+          <t>Saídas do funil</t>
         </is>
       </c>
       <c r="C100" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="D100" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>93</v>
+      </c>
+      <c r="D100" s="22" t="inlineStr">
+        <is>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E100" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Portal Parceiros AIVA → aiva_portal_diario (fonte) → aiva_desempenho (mês/semana)</t>
+          <t>Lojas menos de 01 Ano (automação 101): CNPJ &lt; 1 ano na Receita → NAO_QUALIFICADO (regra 08/09)</t>
         </is>
       </c>
       <c r="G100" s="4" t="inlineStr"/>
@@ -4554,27 +4550,27 @@
     </row>
     <row r="101">
       <c r="A101" s="4" t="n">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Loja Finalizada e Vendendo</t>
+          <t>Saídas do funil</t>
         </is>
       </c>
       <c r="C101" s="4" t="n">
-        <v>51</v>
-      </c>
-      <c r="D101" s="21" t="inlineStr">
-        <is>
-          <t>Sistemas e dados</t>
+        <v>19</v>
+      </c>
+      <c r="D101" s="22" t="inlineStr">
+        <is>
+          <t>Saída</t>
         </is>
       </c>
       <c r="E101" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>sdr_repasses_solicitados → planilha Repasses · contas MRR no Evo</t>
+          <t>Funil 19 · Odres / UME (transferência): CNPJ já na base AIVA/Odres → mensagem oficial + tag ODRES/UME · sdr_leads apaga o lead</t>
         </is>
       </c>
       <c r="G101" s="4" t="inlineStr"/>
@@ -4590,20 +4586,18 @@
           <t>Saídas do funil</t>
         </is>
       </c>
-      <c r="C102" s="4" t="n">
-        <v>53</v>
-      </c>
+      <c r="C102" s="4" t="inlineStr"/>
       <c r="D102" s="22" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
       <c r="E102" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Interessado (Sem resposta) (automação 98): auto-descarte (Início +15d) · régua-saída · SEM_RESPOSTA +30d → DESCARTADO</t>
+          <t>OPT_OUT · LGPD (webhook): "não quero mais" → OPT_OUT · pedido de exclusão → confirma, apaga dados, guarda só o telefone</t>
         </is>
       </c>
       <c r="G102" s="4" t="inlineStr"/>
@@ -4619,20 +4613,18 @@
           <t>Saídas do funil</t>
         </is>
       </c>
-      <c r="C103" s="4" t="n">
-        <v>69</v>
-      </c>
+      <c r="C103" s="4" t="inlineStr"/>
       <c r="D103" s="22" t="inlineStr">
         <is>
           <t>Saída</t>
         </is>
       </c>
       <c r="E103" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F103" s="4" t="inlineStr">
         <is>
-          <t>Bot Detectado (automação 100): VictorIA detectou auto-resposta; reativação recomeça do zero</t>
+          <t>DESCARTADO / NAO_QUALIFICADO (terminal): Descarte manual do Nei é respeitado; status terminais nunca são revividos pelo sync</t>
         </is>
       </c>
       <c r="G103" s="4" t="inlineStr"/>
@@ -4641,27 +4633,25 @@
     </row>
     <row r="104">
       <c r="A104" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Saídas do funil</t>
-        </is>
-      </c>
-      <c r="C104" s="4" t="n">
-        <v>93</v>
-      </c>
-      <c r="D104" s="22" t="inlineStr">
-        <is>
-          <t>Saída</t>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr"/>
+      <c r="D104" s="23" t="inlineStr">
+        <is>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="E104" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>Lojas menos de 01 Ano (automação 101): CNPJ &lt; 1 ano na Receita → NAO_QUALIFICADO (regra 08/09)</t>
+          <t>🔁 Sincronização Evo ↔ painel: Cada etapa tem uma automação de entrada que chama /opportunity-stage (≈1 s). Reforço: sync-from-evo a cada 5 min, Evo é a fonte da verdade (exceções: descarte manual, terminais, guarda de 2 min).</t>
         </is>
       </c>
       <c r="G104" s="4" t="inlineStr"/>
@@ -4670,27 +4660,25 @@
     </row>
     <row r="105">
       <c r="A105" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Saídas do funil</t>
-        </is>
-      </c>
-      <c r="C105" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="D105" s="22" t="inlineStr">
-        <is>
-          <t>Saída</t>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="C105" s="4" t="inlineStr"/>
+      <c r="D105" s="23" t="inlineStr">
+        <is>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="E105" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F105" s="4" t="inlineStr">
         <is>
-          <t>Funil 19 · Odres / UME (transferência): CNPJ já na base AIVA/Odres → mensagem oficial + tag ODRES/UME · sdr_leads apaga o lead</t>
+          <t>🛠 Auto-reprocess (10 min): Mensagem do lead sem resposta da VictorIA → reprocessa; falha da Claude → até N tentativas e depois escala humano.</t>
         </is>
       </c>
       <c r="G105" s="4" t="inlineStr"/>
@@ -4699,25 +4687,25 @@
     </row>
     <row r="106">
       <c r="A106" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Saídas do funil</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr"/>
-      <c r="D106" s="22" t="inlineStr">
-        <is>
-          <t>Saída</t>
+      <c r="D106" s="23" t="inlineStr">
+        <is>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="E106" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>OPT_OUT · LGPD (webhook): "não quero mais" → OPT_OUT · pedido de exclusão → confirma, apaga dados, guarda só o telefone</t>
+          <t>👤 Fila humana: acionar_humano=true entra na fila: 🔴 ação · 📄 docs · 🟡 mover card. WhatsApp pro Nei 8h seg–sex + painel /atendimento (chamados, CS, travados, CNPJ).</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr"/>
@@ -4726,25 +4714,25 @@
     </row>
     <row r="107">
       <c r="A107" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Saídas do funil</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr"/>
-      <c r="D107" s="22" t="inlineStr">
-        <is>
-          <t>Saída</t>
+      <c r="D107" s="23" t="inlineStr">
+        <is>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="E107" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F107" s="4" t="inlineStr">
         <is>
-          <t>DESCARTADO / NAO_QUALIFICADO (terminal): Descarte manual do Nei é respeitado; status terminais nunca são revividos pelo sync</t>
+          <t>📋 Chamados: Erro relatado → pede print → sdr_chamados + planilha Chamados. Nei clica Resolver → planilha recebe "sim" e o chamado some.</t>
         </is>
       </c>
       <c r="G107" s="4" t="inlineStr"/>
@@ -4767,11 +4755,11 @@
         </is>
       </c>
       <c r="E108" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>🔁 Sincronização Evo ↔ painel: Cada etapa tem uma automação de entrada que chama /opportunity-stage (≈1 s). Reforço: sync-from-evo a cada 5 min, Evo é a fonte da verdade (exceções: descarte manual, terminais, guarda de 2 min).</t>
+          <t>📣 Alertas: Transições de status alertam Nei/Aldo via WhatsApp (pré-aprovação, cadastro ✅, CAF confirmado, loja sem operar, contato a confirmar).</t>
         </is>
       </c>
       <c r="G108" s="4" t="inlineStr"/>
@@ -4794,11 +4782,11 @@
         </is>
       </c>
       <c r="E109" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F109" s="4" t="inlineStr">
         <is>
-          <t>🛠 Auto-reprocess (10 min): Mensagem do lead sem resposta da VictorIA → reprocessa; falha da Claude → até N tentativas e depois escala humano.</t>
+          <t>📰 Briefings: briefing-pipeline 5h seg–sex (Aldo + Nei) · auditoria Evo × Supabase (só alerta) · destilador semanal sex 10h (curadoria).</t>
         </is>
       </c>
       <c r="G109" s="4" t="inlineStr"/>
@@ -4821,11 +4809,11 @@
         </is>
       </c>
       <c r="E110" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>👤 Fila humana: acionar_humano=true entra na fila: 🔴 ação · 📄 docs · 🟡 mover card. WhatsApp pro Nei 8h seg–sex + painel /atendimento (chamados, CS, travados, CNPJ).</t>
+          <t>🧠 VictorIA Analista: Widget do painel: consulta leads, conversas, chamados, repasses, desempenho semanal e curadoria. Só leitura.</t>
         </is>
       </c>
       <c r="G110" s="4" t="inlineStr"/>
@@ -4848,129 +4836,21 @@
         </is>
       </c>
       <c r="E111" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F111" s="4" t="inlineStr">
         <is>
-          <t>📋 Chamados: Erro relatado → pede print → sdr_chamados + planilha Chamados. Nei clica Resolver → planilha recebe "sim" e o chamado some.</t>
+          <t>🗓 Data injetada a cada turno: A VictorIA não sabe o dia — lib/claude.ts injeta a data BRT fora do cache. Feriados/avisos entram como bloco dinâmico.</t>
         </is>
       </c>
       <c r="G111" s="4" t="inlineStr"/>
       <c r="H111" s="4" t="inlineStr"/>
       <c r="I111" s="4" t="inlineStr"/>
     </row>
-    <row r="112">
-      <c r="A112" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B112" s="4" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="C112" s="4" t="inlineStr"/>
-      <c r="D112" s="23" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F112" s="4" t="inlineStr">
-        <is>
-          <t>📣 Alertas: Transições de status alertam Nei/Aldo via WhatsApp (pré-aprovação, cadastro ✅, CAF confirmado, loja sem operar, contato a confirmar).</t>
-        </is>
-      </c>
-      <c r="G112" s="4" t="inlineStr"/>
-      <c r="H112" s="4" t="inlineStr"/>
-      <c r="I112" s="4" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="C113" s="4" t="inlineStr"/>
-      <c r="D113" s="23" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>📰 Briefings: briefing-pipeline 5h seg–sex (Aldo + Nei) · auditoria Evo × Supabase (só alerta) · destilador semanal sex 10h (curadoria).</t>
-        </is>
-      </c>
-      <c r="G113" s="4" t="inlineStr"/>
-      <c r="H113" s="4" t="inlineStr"/>
-      <c r="I113" s="4" t="inlineStr"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B114" s="4" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="C114" s="4" t="inlineStr"/>
-      <c r="D114" s="23" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="E114" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F114" s="4" t="inlineStr">
-        <is>
-          <t>🧠 VictorIA Analista: Widget do painel: consulta leads, conversas, chamados, repasses, desempenho semanal e curadoria. Só leitura.</t>
-        </is>
-      </c>
-      <c r="G114" s="4" t="inlineStr"/>
-      <c r="H114" s="4" t="inlineStr"/>
-      <c r="I114" s="4" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B115" s="4" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="C115" s="4" t="inlineStr"/>
-      <c r="D115" s="23" t="inlineStr">
-        <is>
-          <t>Transversal</t>
-        </is>
-      </c>
-      <c r="E115" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F115" s="4" t="inlineStr">
-        <is>
-          <t>🗓 Data injetada a cada turno: A VictorIA não sabe o dia — lib/claude.ts injeta a data BRT fora do cache. Feriados/avisos entram como bloco dinâmico.</t>
-        </is>
-      </c>
-      <c r="G115" s="4" t="inlineStr"/>
-      <c r="H115" s="4" t="inlineStr"/>
-      <c r="I115" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I115"/>
+  <autoFilter ref="A1:I111"/>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G115" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G111" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"sim,não,mudar"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5318,7 +5198,7 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>auto-descarte (Início +15d) · régua-saída · SEM_RESPOSTA +30d → DESCARTADO</t>
+          <t>auto-descarte (Início +15d) · SEM_RESPOSTA +30d → DESCARTADO</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr"/>

</xml_diff>